<commit_message>
fix(salesforce): map Site to sitetracker__Site__c for Sitetracker managed package
</commit_message>
<xml_diff>
--- a/data/common/Mapping_file.xlsx
+++ b/data/common/Mapping_file.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -533,7 +533,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -571,7 +571,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -639,7 +639,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -673,7 +673,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -711,7 +711,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -745,7 +745,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -825,7 +825,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -863,7 +863,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -901,7 +901,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -981,7 +981,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>

</xml_diff>